<commit_message>
Complete Milestone 3 AI career assistance and documentation
</commit_message>
<xml_diff>
--- a/documentation/Copy of Defect_Tracker Template_v0.1.xlsx
+++ b/documentation/Copy of Defect_Tracker Template_v0.1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0ba97a91002e3819/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0ba97a91002e3819/Documents/AI-Career-companion-Agent/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94BFADEF-A1AF-4DC1-85D3-9A5558650627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="8_{94BFADEF-A1AF-4DC1-85D3-9A5558650627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55E917CB-FEDD-4CF8-9FCB-3FCE42BD5D8B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
   <si>
     <t>Sl No</t>
   </si>
@@ -69,13 +69,55 @@
   </si>
   <si>
     <t>Status(Open/Closed)</t>
+  </si>
+  <si>
+    <t>Dharma Teja</t>
+  </si>
+  <si>
+    <t>Mock interview page generated a BuildError because the mock interview route was not defined correctly</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Added and corrected the mock interview route and URL mapping.</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>Mock interview page opened successfully after the route was corrected.</t>
+  </si>
+  <si>
+    <t>Mock interview encountered an undefined m3_mock_interview_agent reference.</t>
+  </si>
+  <si>
+    <t>Corrected the agent initialization and reference in the application.</t>
+  </si>
+  <si>
+    <t>Mock interview agent loaded correctly.</t>
+  </si>
+  <si>
+    <t>Mock interview stopped during the session because conversation state exceeded the normal Flask session storage behavior.</t>
+  </si>
+  <si>
+    <t>Integration</t>
+  </si>
+  <si>
+    <t>Configured Flask-Session and corrected session storage for mock interview state.</t>
+  </si>
+  <si>
+    <t>Mock interview continued correctly across multiple questions.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -132,6 +174,10 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -174,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -191,6 +237,17 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,7 +553,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K20"/>
-  <sheetFormatPr defaultColWidth="17.5546875" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="17.5546875" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="6.109375" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.44140625" style="4" bestFit="1" customWidth="1"/>
@@ -510,7 +567,7 @@
     <col min="12" max="16384" width="17.5546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="31.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -545,49 +602,121 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-    </row>
-    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-    </row>
-    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+    <row r="2" spans="1:11" ht="66.599999999999994">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="8">
+        <v>46282</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="8">
+        <v>46282</v>
+      </c>
+      <c r="J2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="53.4">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="8">
+        <v>46282</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="12">
+        <v>46282</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="53.4">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="12">
+        <v>46283</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="12">
+        <v>46283</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15.6">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="12">
+        <v>46284</v>
+      </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -597,7 +726,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15.6">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -610,7 +739,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15.6">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -623,7 +752,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15.6">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -636,7 +765,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="15.6">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -649,7 +778,7 @@
       <c r="J9" s="3"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="15.6">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -662,7 +791,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15.6">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -675,7 +804,7 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="15.6">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -688,7 +817,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15.6">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -701,7 +830,7 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="15.6">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -714,7 +843,7 @@
       <c r="J14" s="3"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="15.6">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -727,7 +856,7 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="15.6">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -740,7 +869,7 @@
       <c r="J16" s="3"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="15.6">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -753,7 +882,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="15.6">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -766,7 +895,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="15.6">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -779,7 +908,7 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15.6">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -804,7 +933,7 @@
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>G1:G1048576</xm:sqref>
+          <xm:sqref>G1 G5:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -815,29 +944,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1">
       <c r="A5" s="7" t="s">
         <v>14</v>
       </c>
@@ -849,9 +978,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -987,19 +1119,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1023,9 +1151,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Complete AI Career Companion project and documentation
</commit_message>
<xml_diff>
--- a/documentation/Copy of Defect_Tracker Template_v0.1.xlsx
+++ b/documentation/Copy of Defect_Tracker Template_v0.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0ba97a91002e3819/Documents/AI-Career-companion-Agent/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{94BFADEF-A1AF-4DC1-85D3-9A5558650627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55E917CB-FEDD-4CF8-9FCB-3FCE42BD5D8B}"/>
+  <xr:revisionPtr revIDLastSave="109" documentId="8_{94BFADEF-A1AF-4DC1-85D3-9A5558650627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2E84198-94C5-490F-ABC1-A83D3AB3AF9B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="43">
   <si>
     <t>Sl No</t>
   </si>
@@ -111,6 +111,63 @@
   </si>
   <si>
     <t>Mock interview continued correctly across multiple questions.</t>
+  </si>
+  <si>
+    <t>Interview preparation guidance and skill-gap preparation were displayed as raw Python dictionary values instead of formatted information.</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>Updated the Jinja template to display dictionary fields such as category, action, gap, status and preparation method separately.</t>
+  </si>
+  <si>
+    <t>Preparation guidance and skill-gap preparation are now displayed clearly.</t>
+  </si>
+  <si>
+    <t>Application record was not saved correctly after submission.</t>
+  </si>
+  <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Enter how you actually fixed it; if not fixed yet, write </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Pending investigation and correction.</t>
+    </r>
+  </si>
+  <si>
+    <t>Describe the actual test result or remaining issue</t>
+  </si>
+  <si>
+    <t>Application status was not updated correctly after selecting a new status</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Describe the correction, or write </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Pending investigation and correction.</t>
+    </r>
+  </si>
+  <si>
+    <t>Record the actual retest result or explain why the issue remains open.</t>
+  </si>
+  <si>
+    <t>Application records were not displayed correctly in the application tracking interface.</t>
+  </si>
+  <si>
+    <t>Record whether the records displayed correctly after retesting.</t>
   </si>
 </sst>
 </file>
@@ -707,7 +764,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.6">
+    <row r="5" spans="1:11" ht="79.8">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -717,53 +774,135 @@
       <c r="C5" s="12">
         <v>46284</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.6">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.6">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="6"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.6">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
+      <c r="D5" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" s="12">
+        <v>46284</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="66.599999999999994">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="12">
+        <v>46289</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
+        <v>19</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="12">
+        <v>46290</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="66.599999999999994">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="12">
+        <v>46293</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="12">
+        <v>46294</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="53.4">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="12">
+        <v>46297</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="12">
+        <v>46298</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="9" spans="1:11" ht="15.6">
       <c r="A9" s="5"/>
@@ -933,7 +1072,7 @@
           <x14:formula1>
             <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>G1 G5:G1048576</xm:sqref>
+          <xm:sqref>G1 G9:G1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -978,12 +1117,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1119,15 +1255,19 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1151,10 +1291,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>